<commit_message>
UK daily ratings for 2026-06-21
</commit_message>
<xml_diff>
--- a/output/daily_ratings/uk_ratings_2026-06-21.xlsx
+++ b/output/daily_ratings/uk_ratings_2026-06-21.xlsx
@@ -653,7 +653,7 @@
         <v>9</v>
       </c>
       <c r="J4" t="n">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="K4" t="n">
         <v>51</v>
@@ -665,7 +665,7 @@
         <v>95.53</v>
       </c>
       <c r="N4" t="n">
-        <v>49.1</v>
+        <v>42.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         <v>4</v>
       </c>
       <c r="J5" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="K5" t="n">
         <v>70</v>
@@ -725,7 +725,7 @@
         <v>95.53</v>
       </c>
       <c r="N5" t="n">
-        <v>51.3</v>
+        <v>45.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         <v>5</v>
       </c>
       <c r="J6" t="n">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="K6" t="n">
         <v>57</v>
@@ -785,7 +785,7 @@
         <v>95.53</v>
       </c>
       <c r="N6" t="n">
-        <v>41.9</v>
+        <v>39.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -833,7 +833,7 @@
         <v>9</v>
       </c>
       <c r="J7" t="n">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K7" t="n">
         <v>52</v>
@@ -845,7 +845,7 @@
         <v>95.53</v>
       </c>
       <c r="N7" t="n">
-        <v>34</v>
+        <v>28.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1778,34 +1778,36 @@
         <v>6</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Twilight Guest</t>
+          <t>Lucky Sevens</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="K23" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>121.54</v>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="n">
+        <v>51.7</v>
+      </c>
       <c r="O23" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>-5.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1834,34 +1836,38 @@
         <v>6</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Rockafeller Skank (IRE)</t>
+          <t>Dogged</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J24" t="n">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="K24" t="n">
-        <v>72</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.15</v>
+      </c>
       <c r="M24" t="n">
         <v>121.54</v>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="n">
+        <v>47.7</v>
+      </c>
       <c r="O24" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P24" t="n">
-        <v>-5.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1890,28 +1896,30 @@
         <v>6</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Lucky Sevens</t>
+          <t>West Hill Rosie</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J25" t="n">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="K25" t="n">
-        <v>54</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
+        <v>55</v>
+      </c>
+      <c r="L25" t="n">
+        <v>8.15</v>
+      </c>
       <c r="M25" t="n">
         <v>121.54</v>
       </c>
       <c r="N25" t="n">
-        <v>51.7</v>
+        <v>40.7</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -1948,30 +1956,30 @@
         <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Dogged</t>
+          <t>Masqool (IRE)</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J26" t="n">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="K26" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="L26" t="n">
-        <v>0.15</v>
+        <v>9.65</v>
       </c>
       <c r="M26" t="n">
         <v>121.54</v>
       </c>
       <c r="N26" t="n">
-        <v>47.7</v>
+        <v>35.1</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2007,40 +2015,24 @@
       <c r="F27" t="n">
         <v>6</v>
       </c>
-      <c r="G27" t="n">
-        <v>3</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>West Hill Rosie</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>4</v>
-      </c>
-      <c r="J27" t="n">
-        <v>138</v>
-      </c>
-      <c r="K27" t="n">
-        <v>55</v>
-      </c>
-      <c r="L27" t="n">
-        <v>8.15</v>
-      </c>
-      <c r="M27" t="n">
-        <v>121.54</v>
-      </c>
-      <c r="N27" t="n">
-        <v>40.7</v>
-      </c>
+          <t>Twilight Guest</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2067,40 +2059,24 @@
       <c r="F28" t="n">
         <v>6</v>
       </c>
-      <c r="G28" t="n">
-        <v>4</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Masqool (IRE)</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>8</v>
-      </c>
-      <c r="J28" t="n">
-        <v>134</v>
-      </c>
-      <c r="K28" t="n">
-        <v>51</v>
-      </c>
-      <c r="L28" t="n">
-        <v>9.65</v>
-      </c>
-      <c r="M28" t="n">
-        <v>121.54</v>
-      </c>
-      <c r="N28" t="n">
-        <v>35.1</v>
-      </c>
+          <t>Rockafeller Skank (IRE)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2197,7 +2173,7 @@
         <v>3</v>
       </c>
       <c r="J30" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="K30" t="n">
         <v>67</v>
@@ -2209,7 +2185,7 @@
         <v>121.3</v>
       </c>
       <c r="N30" t="n">
-        <v>63.6</v>
+        <v>58.4</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2217,7 +2193,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="31">
@@ -2277,7 +2253,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2555,7 +2531,7 @@
         <v>4</v>
       </c>
       <c r="J36" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K36" t="n">
         <v>60</v>
@@ -2607,7 +2583,7 @@
         <v>3</v>
       </c>
       <c r="J37" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K37" t="n">
         <v>60</v>
@@ -2650,34 +2626,36 @@
         <v>6</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Almavillalobas</t>
+          <t>Shes Got The Blues (IRE)</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J38" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="K38" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="n">
         <v>81.70999999999999</v>
       </c>
-      <c r="N38" t="inlineStr"/>
+      <c r="N38" t="n">
+        <v>57.6</v>
+      </c>
       <c r="O38" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P38" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2706,34 +2684,38 @@
         <v>6</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Fai Fai</t>
+          <t>Spirited Dancer</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J39" t="n">
         <v>135</v>
       </c>
       <c r="K39" t="n">
-        <v>47</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
+        <v>48</v>
+      </c>
+      <c r="L39" t="n">
+        <v>2.75</v>
+      </c>
       <c r="M39" t="n">
         <v>81.70999999999999</v>
       </c>
-      <c r="N39" t="inlineStr"/>
+      <c r="N39" t="n">
+        <v>53.5</v>
+      </c>
       <c r="O39" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P39" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -2762,34 +2744,38 @@
         <v>6</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Mister Sandman</t>
+          <t>My Boy Jack</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J40" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K40" t="n">
-        <v>50</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
+        <v>42</v>
+      </c>
+      <c r="L40" t="n">
+        <v>5</v>
+      </c>
       <c r="M40" t="n">
         <v>81.70999999999999</v>
       </c>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="n">
+        <v>42.4</v>
+      </c>
       <c r="O40" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P40" t="n">
-        <v>-12</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="41">
@@ -2818,28 +2804,30 @@
         <v>6</v>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Shes Got The Blues (IRE)</t>
+          <t>Barnsnape Boy</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J41" t="n">
         <v>128</v>
       </c>
       <c r="K41" t="n">
-        <v>52</v>
-      </c>
-      <c r="L41" t="inlineStr"/>
+        <v>49</v>
+      </c>
+      <c r="L41" t="n">
+        <v>5.05</v>
+      </c>
       <c r="M41" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N41" t="n">
-        <v>57.6</v>
+        <v>38</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -2847,7 +2835,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="42">
@@ -2876,11 +2864,11 @@
         <v>6</v>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Spirited Dancer</t>
+          <t>My Mate Beattie (IRE)</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -2890,16 +2878,16 @@
         <v>135</v>
       </c>
       <c r="K42" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="L42" t="n">
-        <v>2.75</v>
+        <v>5.8</v>
       </c>
       <c r="M42" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N42" t="n">
-        <v>53.5</v>
+        <v>42.5</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -2907,7 +2895,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -2936,30 +2924,30 @@
         <v>6</v>
       </c>
       <c r="G43" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>My Boy Jack</t>
+          <t>Embarked (IRE)</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J43" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K43" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="L43" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="M43" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N43" t="n">
-        <v>46.3</v>
+        <v>37</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -2996,30 +2984,30 @@
         <v>6</v>
       </c>
       <c r="G44" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Barnsnape Boy</t>
+          <t>Skyolaire</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="K44" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="L44" t="n">
-        <v>5.05</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="M44" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N44" t="n">
-        <v>44.3</v>
+        <v>33.1</v>
       </c>
       <c r="O44" t="inlineStr">
         <is>
@@ -3056,30 +3044,30 @@
         <v>6</v>
       </c>
       <c r="G45" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>My Mate Beattie (IRE)</t>
+          <t>Imthequeenofsheba</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J45" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="K45" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="L45" t="n">
-        <v>5.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="M45" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N45" t="n">
-        <v>42.5</v>
+        <v>30.8</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3116,30 +3104,30 @@
         <v>6</v>
       </c>
       <c r="G46" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Embarked (IRE)</t>
+          <t>Mokata</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J46" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="K46" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L46" t="n">
-        <v>6.8</v>
+        <v>14.8</v>
       </c>
       <c r="M46" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N46" t="n">
-        <v>39</v>
+        <v>12.7</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3176,30 +3164,30 @@
         <v>6</v>
       </c>
       <c r="G47" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Skyolaire</t>
+          <t>She Went Whoosh (IRE)</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J47" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="K47" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L47" t="n">
-        <v>8.300000000000001</v>
+        <v>15.3</v>
       </c>
       <c r="M47" t="n">
         <v>81.70999999999999</v>
       </c>
       <c r="N47" t="n">
-        <v>33.1</v>
+        <v>11</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
@@ -3235,40 +3223,24 @@
       <c r="F48" t="n">
         <v>6</v>
       </c>
-      <c r="G48" t="n">
-        <v>8</v>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Imthequeenofsheba</t>
-        </is>
-      </c>
-      <c r="I48" t="n">
-        <v>3</v>
-      </c>
-      <c r="J48" t="n">
-        <v>126</v>
-      </c>
-      <c r="K48" t="n">
-        <v>41</v>
-      </c>
-      <c r="L48" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="M48" t="n">
-        <v>81.70999999999999</v>
-      </c>
-      <c r="N48" t="n">
-        <v>30.8</v>
-      </c>
+          <t>Fai Fai</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P48" t="n">
-        <v>0</v>
-      </c>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3295,40 +3267,24 @@
       <c r="F49" t="n">
         <v>6</v>
       </c>
-      <c r="G49" t="n">
-        <v>9</v>
-      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Mokata</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>3</v>
-      </c>
-      <c r="J49" t="n">
-        <v>126</v>
-      </c>
-      <c r="K49" t="n">
-        <v>46</v>
-      </c>
-      <c r="L49" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="M49" t="n">
-        <v>81.70999999999999</v>
-      </c>
-      <c r="N49" t="n">
-        <v>12.7</v>
-      </c>
+          <t>Mister Sandman</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P49" t="n">
-        <v>0</v>
-      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3355,40 +3311,24 @@
       <c r="F50" t="n">
         <v>6</v>
       </c>
-      <c r="G50" t="n">
-        <v>10</v>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>She Went Whoosh (IRE)</t>
-        </is>
-      </c>
-      <c r="I50" t="n">
-        <v>4</v>
-      </c>
-      <c r="J50" t="n">
-        <v>135</v>
-      </c>
-      <c r="K50" t="n">
-        <v>45</v>
-      </c>
-      <c r="L50" t="n">
-        <v>15.3</v>
-      </c>
-      <c r="M50" t="n">
-        <v>81.70999999999999</v>
-      </c>
-      <c r="N50" t="n">
-        <v>11</v>
-      </c>
+          <t>Almavillalobas</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
       <c r="O50" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P50" t="n">
-        <v>0</v>
-      </c>
+      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3445,7 +3385,7 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3485,7 +3425,7 @@
         <v>6</v>
       </c>
       <c r="J52" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="K52" t="n">
         <v>82</v>
@@ -3497,7 +3437,7 @@
         <v>60.95</v>
       </c>
       <c r="N52" t="n">
-        <v>70.2</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3505,7 +3445,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3545,7 +3485,7 @@
         <v>4</v>
       </c>
       <c r="J53" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="K53" t="n">
         <v>72</v>
@@ -3557,7 +3497,7 @@
         <v>60.95</v>
       </c>
       <c r="N53" t="n">
-        <v>56.9</v>
+        <v>51.7</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -3725,7 +3665,7 @@
         <v>4</v>
       </c>
       <c r="J56" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="K56" t="n">
         <v>68</v>
@@ -3737,7 +3677,7 @@
         <v>60.95</v>
       </c>
       <c r="N56" t="n">
-        <v>21.3</v>
+        <v>17.4</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -4132,34 +4072,36 @@
         <v>6</v>
       </c>
       <c r="G63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>One Of Our Own</t>
+          <t>Instant Bond</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J63" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="K63" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="n">
         <v>75.67</v>
       </c>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="n">
+        <v>63.9</v>
+      </c>
       <c r="O63" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P63" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -4188,28 +4130,30 @@
         <v>6</v>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Instant Bond</t>
+          <t>Melissa Honey</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="K64" t="n">
-        <v>57</v>
-      </c>
-      <c r="L64" t="inlineStr"/>
+        <v>53</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.5</v>
+      </c>
       <c r="M64" t="n">
         <v>75.67</v>
       </c>
       <c r="N64" t="n">
-        <v>63.9</v>
+        <v>56.6</v>
       </c>
       <c r="O64" t="inlineStr">
         <is>
@@ -4246,30 +4190,30 @@
         <v>6</v>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Melissa Honey</t>
+          <t>Invincible Ruby (IRE)</t>
         </is>
       </c>
       <c r="I65" t="n">
         <v>4</v>
       </c>
       <c r="J65" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="K65" t="n">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="L65" t="n">
-        <v>0.5</v>
+        <v>1.75</v>
       </c>
       <c r="M65" t="n">
         <v>75.67</v>
       </c>
       <c r="N65" t="n">
-        <v>56.6</v>
+        <v>59.1</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -4277,7 +4221,7 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4306,30 +4250,30 @@
         <v>6</v>
       </c>
       <c r="G66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Invincible Ruby (IRE)</t>
+          <t>Ideal Guest (FR)</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J66" t="n">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K66" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="L66" t="n">
-        <v>1.75</v>
+        <v>1.9</v>
       </c>
       <c r="M66" t="n">
         <v>75.67</v>
       </c>
       <c r="N66" t="n">
-        <v>64.09999999999999</v>
+        <v>55.7</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -4337,7 +4281,7 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -4366,30 +4310,30 @@
         <v>6</v>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Ideal Guest (FR)</t>
+          <t>Maui Breeze</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J67" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K67" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L67" t="n">
-        <v>1.9</v>
+        <v>4.4</v>
       </c>
       <c r="M67" t="n">
         <v>75.67</v>
       </c>
       <c r="N67" t="n">
-        <v>55.7</v>
+        <v>52.2</v>
       </c>
       <c r="O67" t="inlineStr">
         <is>
@@ -4426,30 +4370,30 @@
         <v>6</v>
       </c>
       <c r="G68" t="n">
+        <v>6</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Diligent Henry</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
         <v>5</v>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>Maui Breeze</t>
-        </is>
-      </c>
-      <c r="I68" t="n">
-        <v>4</v>
-      </c>
       <c r="J68" t="n">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="K68" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="L68" t="n">
-        <v>4.4</v>
+        <v>4.550000000000001</v>
       </c>
       <c r="M68" t="n">
         <v>75.67</v>
       </c>
       <c r="N68" t="n">
-        <v>52.2</v>
+        <v>40.9</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -4486,30 +4430,30 @@
         <v>6</v>
       </c>
       <c r="G69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Diligent Henry</t>
+          <t>Zivas Star</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J69" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K69" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L69" t="n">
-        <v>4.55</v>
+        <v>6.800000000000001</v>
       </c>
       <c r="M69" t="n">
         <v>75.67</v>
       </c>
       <c r="N69" t="n">
-        <v>40.9</v>
+        <v>32.6</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -4517,7 +4461,7 @@
         </is>
       </c>
       <c r="P69" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="70">
@@ -4546,30 +4490,30 @@
         <v>6</v>
       </c>
       <c r="G70" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Zivas Star</t>
+          <t>Hes An Angel</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J70" t="n">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="K70" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="L70" t="n">
-        <v>6.8</v>
+        <v>7.300000000000001</v>
       </c>
       <c r="M70" t="n">
         <v>75.67</v>
       </c>
       <c r="N70" t="n">
-        <v>32.6</v>
+        <v>39.5</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -4577,7 +4521,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -4606,30 +4550,30 @@
         <v>6</v>
       </c>
       <c r="G71" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Hes An Angel</t>
+          <t>Ishe Worth Agamble</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J71" t="n">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K71" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="L71" t="n">
-        <v>7.3</v>
+        <v>7.35</v>
       </c>
       <c r="M71" t="n">
         <v>75.67</v>
       </c>
       <c r="N71" t="n">
-        <v>39.5</v>
+        <v>40.7</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -4637,7 +4581,7 @@
         </is>
       </c>
       <c r="P71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -4666,30 +4610,30 @@
         <v>6</v>
       </c>
       <c r="G72" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Ishe Worth Agamble</t>
+          <t>So Grateful</t>
         </is>
       </c>
       <c r="I72" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J72" t="n">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="K72" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="L72" t="n">
-        <v>7.35</v>
+        <v>8.850000000000001</v>
       </c>
       <c r="M72" t="n">
         <v>75.67</v>
       </c>
       <c r="N72" t="n">
-        <v>40.7</v>
+        <v>23.2</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -4697,7 +4641,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -4726,30 +4670,30 @@
         <v>6</v>
       </c>
       <c r="G73" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>So Grateful</t>
+          <t>Lindoro</t>
         </is>
       </c>
       <c r="I73" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J73" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="K73" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="L73" t="n">
-        <v>8.85</v>
+        <v>14.85</v>
       </c>
       <c r="M73" t="n">
         <v>75.67</v>
       </c>
       <c r="N73" t="n">
-        <v>29.4</v>
+        <v>21.6</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
@@ -4785,40 +4729,24 @@
       <c r="F74" t="n">
         <v>6</v>
       </c>
-      <c r="G74" t="n">
-        <v>11</v>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Lindoro</t>
-        </is>
-      </c>
-      <c r="I74" t="n">
-        <v>4</v>
-      </c>
-      <c r="J74" t="n">
-        <v>135</v>
-      </c>
-      <c r="K74" t="n">
-        <v>60</v>
-      </c>
-      <c r="L74" t="n">
-        <v>14.85</v>
-      </c>
-      <c r="M74" t="n">
-        <v>75.67</v>
-      </c>
-      <c r="N74" t="n">
-        <v>21.6</v>
-      </c>
+          <t>One Of Our Own</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P74" t="n">
-        <v>0</v>
-      </c>
+      <c r="P74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4846,34 +4774,36 @@
         <v>4</v>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Dakota Gold</t>
+          <t>Equity Law</t>
         </is>
       </c>
       <c r="I75" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J75" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="K75" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="n">
         <v>61.91</v>
       </c>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" t="n">
+        <v>79.40000000000001</v>
+      </c>
       <c r="O75" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P75" t="n">
-        <v>-10</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="76">
@@ -4902,28 +4832,30 @@
         <v>4</v>
       </c>
       <c r="G76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Equity Law</t>
+          <t>Lethal Nymph</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J76" t="n">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="K76" t="n">
-        <v>72</v>
-      </c>
-      <c r="L76" t="inlineStr"/>
+        <v>78</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M76" t="n">
         <v>61.91</v>
       </c>
       <c r="N76" t="n">
-        <v>79.40000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
@@ -4931,7 +4863,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -4960,30 +4892,30 @@
         <v>4</v>
       </c>
       <c r="G77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Lethal Nymph</t>
+          <t>Goyard (IRE)</t>
         </is>
       </c>
       <c r="I77" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J77" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="K77" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="L77" t="n">
-        <v>0.1</v>
+        <v>0.85</v>
       </c>
       <c r="M77" t="n">
         <v>61.91</v>
       </c>
       <c r="N77" t="n">
-        <v>81.90000000000001</v>
+        <v>82.2</v>
       </c>
       <c r="O77" t="inlineStr">
         <is>
@@ -4991,7 +4923,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
@@ -5020,30 +4952,30 @@
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Goyard (IRE)</t>
+          <t>Reigning Profit (IRE)</t>
         </is>
       </c>
       <c r="I78" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J78" t="n">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="K78" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L78" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="M78" t="n">
         <v>61.91</v>
       </c>
       <c r="N78" t="n">
-        <v>82.2</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="O78" t="inlineStr">
         <is>
@@ -5051,7 +4983,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -5080,30 +5012,30 @@
         <v>4</v>
       </c>
       <c r="G79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Reigning Profit (IRE)</t>
+          <t>D Flawless (IRE)</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J79" t="n">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="K79" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L79" t="n">
-        <v>0.95</v>
+        <v>1.7</v>
       </c>
       <c r="M79" t="n">
         <v>61.91</v>
       </c>
       <c r="N79" t="n">
-        <v>78.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
@@ -5111,7 +5043,7 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="80">
@@ -5140,15 +5072,15 @@
         <v>4</v>
       </c>
       <c r="G80" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>D Flawless (IRE)</t>
+          <t>Ventura Express</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J80" t="n">
         <v>128</v>
@@ -5157,13 +5089,13 @@
         <v>73</v>
       </c>
       <c r="L80" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="M80" t="n">
         <v>61.91</v>
       </c>
       <c r="N80" t="n">
-        <v>71.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="O80" t="inlineStr">
         <is>
@@ -5200,30 +5132,30 @@
         <v>4</v>
       </c>
       <c r="G81" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Ventura Express</t>
+          <t>Hiya Maite</t>
         </is>
       </c>
       <c r="I81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J81" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K81" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="L81" t="n">
-        <v>1.8</v>
+        <v>2.55</v>
       </c>
       <c r="M81" t="n">
         <v>61.91</v>
       </c>
       <c r="N81" t="n">
-        <v>69.90000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="O81" t="inlineStr">
         <is>
@@ -5231,7 +5163,7 @@
         </is>
       </c>
       <c r="P81" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -5260,30 +5192,30 @@
         <v>4</v>
       </c>
       <c r="G82" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Hiya Maite</t>
+          <t>Squealer (IRE)</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J82" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="K82" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="L82" t="n">
-        <v>2.55</v>
+        <v>3.05</v>
       </c>
       <c r="M82" t="n">
         <v>61.91</v>
       </c>
       <c r="N82" t="n">
-        <v>74.7</v>
+        <v>68.8</v>
       </c>
       <c r="O82" t="inlineStr">
         <is>
@@ -5291,7 +5223,7 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -5320,30 +5252,30 @@
         <v>4</v>
       </c>
       <c r="G83" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Squealer (IRE)</t>
+          <t>South Parade (IRE)</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J83" t="n">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="K83" t="n">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="L83" t="n">
-        <v>3.05</v>
+        <v>14.05</v>
       </c>
       <c r="M83" t="n">
         <v>61.91</v>
       </c>
       <c r="N83" t="n">
-        <v>68.8</v>
+        <v>21.8</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -5379,40 +5311,24 @@
       <c r="F84" t="n">
         <v>4</v>
       </c>
-      <c r="G84" t="n">
-        <v>9</v>
-      </c>
+      <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>South Parade (IRE)</t>
-        </is>
-      </c>
-      <c r="I84" t="n">
-        <v>5</v>
-      </c>
-      <c r="J84" t="n">
-        <v>118</v>
-      </c>
-      <c r="K84" t="n">
-        <v>63</v>
-      </c>
-      <c r="L84" t="n">
-        <v>14.05</v>
-      </c>
-      <c r="M84" t="n">
-        <v>61.91</v>
-      </c>
-      <c r="N84" t="n">
-        <v>21.8</v>
-      </c>
+          <t>Dakota Gold</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P84" t="n">
-        <v>0</v>
-      </c>
+      <c r="P84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5440,34 +5356,36 @@
         <v>1</v>
       </c>
       <c r="G85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Ryka (IRE)</t>
+          <t>Coedana (IRE)</t>
         </is>
       </c>
       <c r="I85" t="n">
         <v>4</v>
       </c>
       <c r="J85" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K85" t="n">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="n">
         <v>153.97</v>
       </c>
-      <c r="N85" t="inlineStr"/>
+      <c r="N85" t="n">
+        <v>100.2</v>
+      </c>
       <c r="O85" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P85" t="n">
-        <v>-10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -5496,11 +5414,11 @@
         <v>1</v>
       </c>
       <c r="G86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Coedana (IRE)</t>
+          <t>Revoir</t>
         </is>
       </c>
       <c r="I86" t="n">
@@ -5510,14 +5428,16 @@
         <v>128</v>
       </c>
       <c r="K86" t="n">
-        <v>103</v>
-      </c>
-      <c r="L86" t="inlineStr"/>
+        <v>101</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0.15</v>
+      </c>
       <c r="M86" t="n">
         <v>153.97</v>
       </c>
       <c r="N86" t="n">
-        <v>100.2</v>
+        <v>98.8</v>
       </c>
       <c r="O86" t="inlineStr">
         <is>
@@ -5554,30 +5474,30 @@
         <v>1</v>
       </c>
       <c r="G87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Revoir</t>
+          <t>Lemsairbat (FR)</t>
         </is>
       </c>
       <c r="I87" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J87" t="n">
         <v>128</v>
       </c>
       <c r="K87" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="L87" t="n">
-        <v>0.15</v>
+        <v>2.4</v>
       </c>
       <c r="M87" t="n">
         <v>153.97</v>
       </c>
       <c r="N87" t="n">
-        <v>98.8</v>
+        <v>93.7</v>
       </c>
       <c r="O87" t="inlineStr">
         <is>
@@ -5614,30 +5534,30 @@
         <v>1</v>
       </c>
       <c r="G88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>Lemsairbat (FR)</t>
+          <t>Merveilleux Lapin (IRE)</t>
         </is>
       </c>
       <c r="I88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J88" t="n">
         <v>128</v>
       </c>
       <c r="K88" t="n">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="L88" t="n">
-        <v>2.4</v>
+        <v>3.65</v>
       </c>
       <c r="M88" t="n">
         <v>153.97</v>
       </c>
       <c r="N88" t="n">
-        <v>93.7</v>
+        <v>90.7</v>
       </c>
       <c r="O88" t="inlineStr">
         <is>
@@ -5674,11 +5594,11 @@
         <v>1</v>
       </c>
       <c r="G89" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Merveilleux Lapin (IRE)</t>
+          <t>Little Dorrit</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -5691,13 +5611,13 @@
         <v>96</v>
       </c>
       <c r="L89" t="n">
-        <v>3.65</v>
+        <v>3.8</v>
       </c>
       <c r="M89" t="n">
         <v>153.97</v>
       </c>
       <c r="N89" t="n">
-        <v>90.7</v>
+        <v>90</v>
       </c>
       <c r="O89" t="inlineStr">
         <is>
@@ -5734,11 +5654,11 @@
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Little Dorrit</t>
+          <t>Brielle</t>
         </is>
       </c>
       <c r="I90" t="n">
@@ -5748,16 +5668,16 @@
         <v>128</v>
       </c>
       <c r="K90" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="L90" t="n">
-        <v>3.8</v>
+        <v>4.550000000000001</v>
       </c>
       <c r="M90" t="n">
         <v>153.97</v>
       </c>
       <c r="N90" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="O90" t="inlineStr">
         <is>
@@ -5794,11 +5714,11 @@
         <v>1</v>
       </c>
       <c r="G91" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Brielle</t>
+          <t>Orionis</t>
         </is>
       </c>
       <c r="I91" t="n">
@@ -5808,16 +5728,16 @@
         <v>128</v>
       </c>
       <c r="K91" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="L91" t="n">
-        <v>4.55</v>
+        <v>5.050000000000001</v>
       </c>
       <c r="M91" t="n">
         <v>153.97</v>
       </c>
       <c r="N91" t="n">
-        <v>88</v>
+        <v>85.3</v>
       </c>
       <c r="O91" t="inlineStr">
         <is>
@@ -5854,11 +5774,11 @@
         <v>1</v>
       </c>
       <c r="G92" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Orionis</t>
+          <t>Ghaiyya</t>
         </is>
       </c>
       <c r="I92" t="n">
@@ -5868,16 +5788,16 @@
         <v>128</v>
       </c>
       <c r="K92" t="n">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L92" t="n">
-        <v>5.05</v>
+        <v>12.55</v>
       </c>
       <c r="M92" t="n">
         <v>153.97</v>
       </c>
       <c r="N92" t="n">
-        <v>85.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="O92" t="inlineStr">
         <is>
@@ -5914,30 +5834,30 @@
         <v>1</v>
       </c>
       <c r="G93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Ghaiyya</t>
+          <t>Cabrera (IRE)</t>
         </is>
       </c>
       <c r="I93" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J93" t="n">
         <v>128</v>
       </c>
       <c r="K93" t="n">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="L93" t="n">
-        <v>12.55</v>
+        <v>13.3</v>
       </c>
       <c r="M93" t="n">
         <v>153.97</v>
       </c>
       <c r="N93" t="n">
-        <v>75.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -5973,40 +5893,24 @@
       <c r="F94" t="n">
         <v>1</v>
       </c>
-      <c r="G94" t="n">
-        <v>9</v>
-      </c>
+      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Cabrera (IRE)</t>
-        </is>
-      </c>
-      <c r="I94" t="n">
-        <v>5</v>
-      </c>
-      <c r="J94" t="n">
-        <v>128</v>
-      </c>
-      <c r="K94" t="n">
-        <v>83</v>
-      </c>
-      <c r="L94" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="M94" t="n">
-        <v>153.97</v>
-      </c>
-      <c r="N94" t="n">
-        <v>73.2</v>
-      </c>
+          <t>Ryka (IRE)</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P94" t="n">
-        <v>0</v>
-      </c>
+      <c r="P94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6034,34 +5938,36 @@
         <v>4</v>
       </c>
       <c r="G95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Treasure Islands</t>
+          <t>Secret Force (IRE)</t>
         </is>
       </c>
       <c r="I95" t="n">
         <v>4</v>
       </c>
       <c r="J95" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K95" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="n">
         <v>247.45</v>
       </c>
-      <c r="N95" t="inlineStr"/>
+      <c r="N95" t="n">
+        <v>-1.4</v>
+      </c>
       <c r="O95" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P95" t="n">
-        <v>-6</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="96">
@@ -6090,28 +5996,30 @@
         <v>4</v>
       </c>
       <c r="G96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Secret Force (IRE)</t>
+          <t>Trojan Soldier</t>
         </is>
       </c>
       <c r="I96" t="n">
         <v>4</v>
       </c>
       <c r="J96" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K96" t="n">
-        <v>74</v>
-      </c>
-      <c r="L96" t="inlineStr"/>
+        <v>78</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0.5</v>
+      </c>
       <c r="M96" t="n">
         <v>247.45</v>
       </c>
       <c r="N96" t="n">
-        <v>-1.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="O96" t="inlineStr">
         <is>
@@ -6119,7 +6027,7 @@
         </is>
       </c>
       <c r="P96" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -6148,30 +6056,30 @@
         <v>4</v>
       </c>
       <c r="G97" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>Trojan Soldier</t>
+          <t>Sax Appeal</t>
         </is>
       </c>
       <c r="I97" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J97" t="n">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="K97" t="n">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="L97" t="n">
-        <v>0.5</v>
+        <v>4.75</v>
       </c>
       <c r="M97" t="n">
         <v>247.45</v>
       </c>
       <c r="N97" t="n">
-        <v>8.800000000000001</v>
+        <v>14.7</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -6179,7 +6087,7 @@
         </is>
       </c>
       <c r="P97" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="98">
@@ -6208,30 +6116,30 @@
         <v>4</v>
       </c>
       <c r="G98" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Sax Appeal</t>
+          <t>Anzac Day (IRE)</t>
         </is>
       </c>
       <c r="I98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J98" t="n">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="K98" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="L98" t="n">
-        <v>4.75</v>
+        <v>5.75</v>
       </c>
       <c r="M98" t="n">
         <v>247.45</v>
       </c>
       <c r="N98" t="n">
-        <v>14.7</v>
+        <v>4.8</v>
       </c>
       <c r="O98" t="inlineStr">
         <is>
@@ -6239,7 +6147,7 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -6268,30 +6176,30 @@
         <v>4</v>
       </c>
       <c r="G99" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Anzac Day (IRE)</t>
+          <t>Isle Of Sark (USA)</t>
         </is>
       </c>
       <c r="I99" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J99" t="n">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="K99" t="n">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="L99" t="n">
-        <v>5.75</v>
+        <v>10.75</v>
       </c>
       <c r="M99" t="n">
         <v>247.45</v>
       </c>
       <c r="N99" t="n">
-        <v>4.8</v>
+        <v>-29.3</v>
       </c>
       <c r="O99" t="inlineStr">
         <is>
@@ -6299,7 +6207,7 @@
         </is>
       </c>
       <c r="P99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -6327,40 +6235,24 @@
       <c r="F100" t="n">
         <v>4</v>
       </c>
-      <c r="G100" t="n">
-        <v>5</v>
-      </c>
+      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Isle Of Sark (USA)</t>
-        </is>
-      </c>
-      <c r="I100" t="n">
-        <v>8</v>
-      </c>
-      <c r="J100" t="n">
-        <v>122</v>
-      </c>
-      <c r="K100" t="n">
-        <v>72</v>
-      </c>
-      <c r="L100" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="M100" t="n">
-        <v>247.45</v>
-      </c>
-      <c r="N100" t="n">
-        <v>-20.2</v>
-      </c>
+          <t>Treasure Islands</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P100" t="n">
-        <v>0</v>
-      </c>
+      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6388,34 +6280,36 @@
         <v>3</v>
       </c>
       <c r="G101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Ray Mon Dough</t>
+          <t>Badri</t>
         </is>
       </c>
       <c r="I101" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J101" t="n">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="K101" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="n">
         <v>75.20999999999999</v>
       </c>
-      <c r="N101" t="inlineStr"/>
+      <c r="N101" t="n">
+        <v>87</v>
+      </c>
       <c r="O101" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P101" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102">
@@ -6444,28 +6338,30 @@
         <v>3</v>
       </c>
       <c r="G102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Badri</t>
+          <t>Rock Opera</t>
         </is>
       </c>
       <c r="I102" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J102" t="n">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="K102" t="n">
-        <v>89</v>
-      </c>
-      <c r="L102" t="inlineStr"/>
+        <v>75</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0.5</v>
+      </c>
       <c r="M102" t="n">
         <v>75.20999999999999</v>
       </c>
       <c r="N102" t="n">
-        <v>87</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="O102" t="inlineStr">
         <is>
@@ -6502,30 +6398,30 @@
         <v>3</v>
       </c>
       <c r="G103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Rock Opera</t>
+          <t>Mister Sox</t>
         </is>
       </c>
       <c r="I103" t="n">
         <v>6</v>
       </c>
       <c r="J103" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K103" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L103" t="n">
-        <v>0.5</v>
+        <v>1.75</v>
       </c>
       <c r="M103" t="n">
         <v>75.20999999999999</v>
       </c>
       <c r="N103" t="n">
-        <v>75.40000000000001</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
@@ -6562,30 +6458,30 @@
         <v>3</v>
       </c>
       <c r="G104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Mister Sox</t>
+          <t>The Good Biscuit</t>
         </is>
       </c>
       <c r="I104" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J104" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="K104" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="L104" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="M104" t="n">
         <v>75.20999999999999</v>
       </c>
       <c r="N104" t="n">
-        <v>70.40000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -6622,30 +6518,30 @@
         <v>3</v>
       </c>
       <c r="G105" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>The Good Biscuit</t>
+          <t>Russet Gold</t>
         </is>
       </c>
       <c r="I105" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J105" t="n">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="K105" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="L105" t="n">
-        <v>2.5</v>
+        <v>5.25</v>
       </c>
       <c r="M105" t="n">
         <v>75.20999999999999</v>
       </c>
       <c r="N105" t="n">
-        <v>69.8</v>
+        <v>68.5</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
@@ -6682,30 +6578,30 @@
         <v>3</v>
       </c>
       <c r="G106" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Russet Gold</t>
+          <t>Azure Zain (FR)</t>
         </is>
       </c>
       <c r="I106" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J106" t="n">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="K106" t="n">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="L106" t="n">
-        <v>5.25</v>
+        <v>8.25</v>
       </c>
       <c r="M106" t="n">
         <v>75.20999999999999</v>
       </c>
       <c r="N106" t="n">
-        <v>68.5</v>
+        <v>49.4</v>
       </c>
       <c r="O106" t="inlineStr">
         <is>
@@ -6741,40 +6637,24 @@
       <c r="F107" t="n">
         <v>3</v>
       </c>
-      <c r="G107" t="n">
-        <v>6</v>
-      </c>
+      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Azure Zain (FR)</t>
-        </is>
-      </c>
-      <c r="I107" t="n">
-        <v>4</v>
-      </c>
-      <c r="J107" t="n">
-        <v>128</v>
-      </c>
-      <c r="K107" t="n">
-        <v>76</v>
-      </c>
-      <c r="L107" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="M107" t="n">
-        <v>75.20999999999999</v>
-      </c>
-      <c r="N107" t="n">
-        <v>53.2</v>
-      </c>
+          <t>Ray Mon Dough</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
       <c r="O107" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="P107" t="n">
-        <v>0</v>
-      </c>
+      <c r="P107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6802,18 +6682,18 @@
         <v>5</v>
       </c>
       <c r="G108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Keep An Eye On It</t>
+          <t>Amidst The Chaos (IRE)</t>
         </is>
       </c>
       <c r="I108" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J108" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="K108" t="n">
         <v>67</v>
@@ -6822,14 +6702,16 @@
       <c r="M108" t="n">
         <v>103.15</v>
       </c>
-      <c r="N108" t="inlineStr"/>
+      <c r="N108" t="n">
+        <v>79.40000000000001</v>
+      </c>
       <c r="O108" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
       <c r="P108" t="n">
-        <v>-8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -6858,28 +6740,30 @@
         <v>5</v>
       </c>
       <c r="G109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Amidst The Chaos (IRE)</t>
+          <t>Gennadius</t>
         </is>
       </c>
       <c r="I109" t="n">
         <v>4</v>
       </c>
       <c r="J109" t="n">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K109" t="n">
-        <v>67</v>
-      </c>
-      <c r="L109" t="inlineStr"/>
+        <v>65</v>
+      </c>
+      <c r="L109" t="n">
+        <v>3.25</v>
+      </c>
       <c r="M109" t="n">
         <v>103.15</v>
       </c>
       <c r="N109" t="n">
-        <v>79.40000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="O109" t="inlineStr">
         <is>
@@ -6916,15 +6800,15 @@
         <v>5</v>
       </c>
       <c r="G110" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Gennadius</t>
+          <t>Ravishing Beauty</t>
         </is>
       </c>
       <c r="I110" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J110" t="n">
         <v>140</v>
@@ -6933,13 +6817,13 @@
         <v>65</v>
       </c>
       <c r="L110" t="n">
-        <v>3.25</v>
+        <v>4.75</v>
       </c>
       <c r="M110" t="n">
         <v>103.15</v>
       </c>
       <c r="N110" t="n">
-        <v>69.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O110" t="inlineStr">
         <is>
@@ -6976,30 +6860,30 @@
         <v>5</v>
       </c>
       <c r="G111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Ravishing Beauty</t>
+          <t>Thats My Boy Luke</t>
         </is>
       </c>
       <c r="I111" t="n">
         <v>5</v>
       </c>
       <c r="J111" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="K111" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="L111" t="n">
-        <v>4.75</v>
+        <v>7</v>
       </c>
       <c r="M111" t="n">
         <v>103.15</v>
       </c>
       <c r="N111" t="n">
-        <v>67.09999999999999</v>
+        <v>57.4</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -7007,7 +6891,7 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="112">
@@ -7036,30 +6920,30 @@
         <v>5</v>
       </c>
       <c r="G112" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Thats My Boy Luke</t>
+          <t>Masaban (IRE)</t>
         </is>
       </c>
       <c r="I112" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J112" t="n">
         <v>135</v>
       </c>
       <c r="K112" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="L112" t="n">
-        <v>7</v>
+        <v>9.25</v>
       </c>
       <c r="M112" t="n">
         <v>103.15</v>
       </c>
       <c r="N112" t="n">
-        <v>57.4</v>
+        <v>58.5</v>
       </c>
       <c r="O112" t="inlineStr">
         <is>
@@ -7067,7 +6951,7 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -7096,30 +6980,30 @@
         <v>5</v>
       </c>
       <c r="G113" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>Masaban (IRE)</t>
+          <t>Mount King (IRE)</t>
         </is>
       </c>
       <c r="I113" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J113" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K113" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="L113" t="n">
-        <v>9.25</v>
+        <v>16.25</v>
       </c>
       <c r="M113" t="n">
         <v>103.15</v>
       </c>
       <c r="N113" t="n">
-        <v>58.5</v>
+        <v>35.3</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -7127,7 +7011,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -7156,34 +7040,34 @@
         <v>5</v>
       </c>
       <c r="G114" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>Mount King (IRE)</t>
+          <t>Kiss For An Angel (IRE)</t>
         </is>
       </c>
       <c r="I114" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J114" t="n">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="K114" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L114" t="n">
-        <v>16.25</v>
+        <v>71.25</v>
       </c>
       <c r="M114" t="n">
         <v>103.15</v>
       </c>
       <c r="N114" t="n">
-        <v>35.3</v>
+        <v>-34.6</v>
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="P114" t="n">
@@ -7215,40 +7099,24 @@
       <c r="F115" t="n">
         <v>5</v>
       </c>
-      <c r="G115" t="n">
-        <v>7</v>
-      </c>
+      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Kiss For An Angel (IRE)</t>
-        </is>
-      </c>
-      <c r="I115" t="n">
-        <v>3</v>
-      </c>
-      <c r="J115" t="n">
-        <v>130</v>
-      </c>
-      <c r="K115" t="n">
-        <v>65</v>
-      </c>
-      <c r="L115" t="n">
-        <v>71.25</v>
-      </c>
-      <c r="M115" t="n">
-        <v>103.15</v>
-      </c>
-      <c r="N115" t="n">
-        <v>-34.6</v>
-      </c>
+          <t>Keep An Eye On It</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr">
         <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="P115" t="n">
-        <v>0</v>
-      </c>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>